<commit_message>
Mise à jour du 03 oct 2026
</commit_message>
<xml_diff>
--- a/HS & COMPLEMENT CSKN.xlsx
+++ b/HS & COMPLEMENT CSKN.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\192.168.1.3\Informatique\DIMONEKENE NSINGI\DONNEES FRANKLIN\FROM VUIDI\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\B.NIMI\Desktop\DIVERS\Fichiers\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5D3CE156-2F3C-4169-9246-D510C323B8EC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CE970697-2834-4AE1-BA67-8BEB194FFD90}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28690" yWindow="-110" windowWidth="29020" windowHeight="15700" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28690" yWindow="-110" windowWidth="29020" windowHeight="15700" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Esprit Sucrière (HS)" sheetId="1" r:id="rId1"/>
@@ -268,9 +268,6 @@
     <t>Notion sur le Complément</t>
   </si>
   <si>
-    <t>Avantage monétaire que laSucrière accorde à ses employés qui ont presté de :</t>
-  </si>
-  <si>
     <t>Pose</t>
   </si>
   <si>
@@ -296,6 +293,9 @@
   </si>
   <si>
     <t>Code Pointage</t>
+  </si>
+  <si>
+    <t>Avantage monétaire que la Sucrière accorde à ses employés qui ont presté de :</t>
   </si>
 </sst>
 </file>
@@ -535,6 +535,12 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="right" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -558,12 +564,6 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -984,7 +984,7 @@
       <c r="F3" s="14">
         <v>12</v>
       </c>
-      <c r="G3" s="39">
+      <c r="G3" s="41">
         <v>36</v>
       </c>
       <c r="H3" s="15">
@@ -1017,7 +1017,7 @@
       <c r="F4" s="14">
         <v>12</v>
       </c>
-      <c r="G4" s="39"/>
+      <c r="G4" s="41"/>
       <c r="H4" s="15">
         <v>4</v>
       </c>
@@ -1048,7 +1048,7 @@
       <c r="F5" s="14">
         <v>12</v>
       </c>
-      <c r="G5" s="39"/>
+      <c r="G5" s="41"/>
       <c r="H5" s="15">
         <v>4</v>
       </c>
@@ -1083,7 +1083,7 @@
       <c r="F6">
         <v>0</v>
       </c>
-      <c r="G6" s="39"/>
+      <c r="G6" s="41"/>
       <c r="H6" s="15"/>
       <c r="I6" s="18" t="s">
         <v>40</v>
@@ -1118,7 +1118,7 @@
       <c r="F7" s="14">
         <v>12</v>
       </c>
-      <c r="G7" s="39">
+      <c r="G7" s="41">
         <v>68</v>
       </c>
       <c r="H7" s="15">
@@ -1157,7 +1157,7 @@
       <c r="F8" s="14">
         <v>12</v>
       </c>
-      <c r="G8" s="39"/>
+      <c r="G8" s="41"/>
       <c r="H8" s="15">
         <v>4</v>
       </c>
@@ -1194,7 +1194,7 @@
       <c r="F9" s="14">
         <v>12</v>
       </c>
-      <c r="G9" s="39"/>
+      <c r="G9" s="41"/>
       <c r="H9" s="15">
         <v>4</v>
       </c>
@@ -1231,7 +1231,7 @@
       <c r="F10" s="14">
         <v>12</v>
       </c>
-      <c r="G10" s="39"/>
+      <c r="G10" s="41"/>
       <c r="H10" s="15">
         <v>4</v>
       </c>
@@ -1268,7 +1268,7 @@
       <c r="F11" s="14">
         <v>12</v>
       </c>
-      <c r="G11" s="39"/>
+      <c r="G11" s="41"/>
       <c r="H11" s="15">
         <v>4</v>
       </c>
@@ -1299,7 +1299,7 @@
       <c r="F12" s="14">
         <v>8</v>
       </c>
-      <c r="G12" s="39"/>
+      <c r="G12" s="41"/>
       <c r="H12" s="15"/>
       <c r="O12" s="5" t="s">
         <v>25</v>
@@ -1355,7 +1355,7 @@
       <c r="F14" s="14">
         <v>8</v>
       </c>
-      <c r="G14" s="39">
+      <c r="G14" s="41">
         <v>48</v>
       </c>
       <c r="I14" s="11" t="s">
@@ -1389,7 +1389,7 @@
       <c r="F15" s="14">
         <v>8</v>
       </c>
-      <c r="G15" s="39"/>
+      <c r="G15" s="41"/>
       <c r="I15" s="11" t="s">
         <v>64</v>
       </c>
@@ -1420,7 +1420,7 @@
       <c r="F16" s="14">
         <v>8</v>
       </c>
-      <c r="G16" s="39"/>
+      <c r="G16" s="41"/>
       <c r="O16" s="5" t="s">
         <v>29</v>
       </c>
@@ -1448,7 +1448,7 @@
       <c r="F17" s="14">
         <v>8</v>
       </c>
-      <c r="G17" s="39"/>
+      <c r="G17" s="41"/>
       <c r="I17" s="17"/>
       <c r="J17" s="19" t="s">
         <v>59</v>
@@ -1489,7 +1489,7 @@
       <c r="F18" s="14">
         <v>8</v>
       </c>
-      <c r="G18" s="39"/>
+      <c r="G18" s="41"/>
       <c r="I18" s="18" t="s">
         <v>58</v>
       </c>
@@ -1532,7 +1532,7 @@
       <c r="F19" s="14">
         <v>8</v>
       </c>
-      <c r="G19" s="39"/>
+      <c r="G19" s="41"/>
       <c r="I19" s="11"/>
       <c r="O19" s="5" t="s">
         <v>32</v>
@@ -1589,10 +1589,10 @@
       <c r="F21" s="14">
         <v>8</v>
       </c>
-      <c r="G21" s="39">
+      <c r="G21" s="41">
         <v>56</v>
       </c>
-      <c r="I21" s="40" t="s">
+      <c r="I21" s="42" t="s">
         <v>62</v>
       </c>
       <c r="J21" s="17">
@@ -1630,8 +1630,8 @@
       <c r="F22" s="14">
         <v>8</v>
       </c>
-      <c r="G22" s="39"/>
-      <c r="I22" s="40"/>
+      <c r="G22" s="41"/>
+      <c r="I22" s="42"/>
       <c r="J22" s="17">
         <v>24</v>
       </c>
@@ -1665,8 +1665,8 @@
       <c r="F23" s="14">
         <v>8</v>
       </c>
-      <c r="G23" s="39"/>
-      <c r="I23" s="40"/>
+      <c r="G23" s="41"/>
+      <c r="I23" s="42"/>
       <c r="J23" s="17">
         <v>36</v>
       </c>
@@ -1700,7 +1700,7 @@
       <c r="F24" s="14">
         <v>8</v>
       </c>
-      <c r="G24" s="39"/>
+      <c r="G24" s="41"/>
       <c r="O24" s="5" t="s">
         <v>10</v>
       </c>
@@ -1728,7 +1728,7 @@
       <c r="F25" s="14">
         <v>12</v>
       </c>
-      <c r="G25" s="39"/>
+      <c r="G25" s="41"/>
       <c r="H25" s="15">
         <v>4</v>
       </c>
@@ -1759,7 +1759,7 @@
       <c r="F26" s="14">
         <v>12</v>
       </c>
-      <c r="G26" s="39"/>
+      <c r="G26" s="41"/>
       <c r="H26" s="15">
         <v>4</v>
       </c>
@@ -2031,7 +2031,7 @@
       <c r="F3" s="14">
         <v>12</v>
       </c>
-      <c r="G3" s="39">
+      <c r="G3" s="41">
         <v>36</v>
       </c>
       <c r="H3" s="15">
@@ -2064,7 +2064,7 @@
       <c r="F4" s="14">
         <v>12</v>
       </c>
-      <c r="G4" s="39"/>
+      <c r="G4" s="41"/>
       <c r="H4" s="15">
         <v>4</v>
       </c>
@@ -2095,7 +2095,7 @@
       <c r="F5" s="14">
         <v>12</v>
       </c>
-      <c r="G5" s="39"/>
+      <c r="G5" s="41"/>
       <c r="H5" s="15">
         <v>7</v>
       </c>
@@ -2124,7 +2124,7 @@
       <c r="F6">
         <v>0</v>
       </c>
-      <c r="G6" s="39"/>
+      <c r="G6" s="41"/>
       <c r="H6" s="15"/>
       <c r="O6" s="5" t="s">
         <v>19</v>
@@ -2153,7 +2153,7 @@
       <c r="F7" s="14">
         <v>12</v>
       </c>
-      <c r="G7" s="39">
+      <c r="G7" s="41">
         <v>68</v>
       </c>
       <c r="H7" s="15">
@@ -2186,7 +2186,7 @@
       <c r="F8" s="14">
         <v>12</v>
       </c>
-      <c r="G8" s="39"/>
+      <c r="G8" s="41"/>
       <c r="H8" s="15">
         <v>4</v>
       </c>
@@ -2217,7 +2217,7 @@
       <c r="F9" s="14">
         <v>12</v>
       </c>
-      <c r="G9" s="39"/>
+      <c r="G9" s="41"/>
       <c r="H9" s="15">
         <v>4</v>
       </c>
@@ -2248,7 +2248,7 @@
       <c r="F10" s="14">
         <v>12</v>
       </c>
-      <c r="G10" s="39"/>
+      <c r="G10" s="41"/>
       <c r="H10" s="15">
         <v>4</v>
       </c>
@@ -2279,7 +2279,7 @@
       <c r="F11" s="14">
         <v>12</v>
       </c>
-      <c r="G11" s="39"/>
+      <c r="G11" s="41"/>
       <c r="H11" s="15">
         <v>4</v>
       </c>
@@ -2310,7 +2310,7 @@
       <c r="F12" s="14">
         <v>8</v>
       </c>
-      <c r="G12" s="39"/>
+      <c r="G12" s="41"/>
       <c r="H12" s="15">
         <v>3</v>
       </c>
@@ -2368,7 +2368,7 @@
       <c r="F14" s="14">
         <v>8</v>
       </c>
-      <c r="G14" s="39">
+      <c r="G14" s="41">
         <v>48</v>
       </c>
       <c r="I14" s="11" t="s">
@@ -2404,7 +2404,7 @@
       <c r="F15" s="14">
         <v>8</v>
       </c>
-      <c r="G15" s="39"/>
+      <c r="G15" s="41"/>
       <c r="O15" s="5" t="s">
         <v>28</v>
       </c>
@@ -2432,7 +2432,7 @@
       <c r="F16" s="14">
         <v>8</v>
       </c>
-      <c r="G16" s="39"/>
+      <c r="G16" s="41"/>
       <c r="O16" s="5" t="s">
         <v>29</v>
       </c>
@@ -2460,7 +2460,7 @@
       <c r="F17" s="14">
         <v>8</v>
       </c>
-      <c r="G17" s="39"/>
+      <c r="G17" s="41"/>
       <c r="J17" s="11" t="s">
         <v>50</v>
       </c>
@@ -2497,7 +2497,7 @@
       <c r="F18" s="14">
         <v>8</v>
       </c>
-      <c r="G18" s="39"/>
+      <c r="G18" s="41"/>
       <c r="I18" s="11" t="s">
         <v>45</v>
       </c>
@@ -2537,7 +2537,7 @@
       <c r="F19" s="14">
         <v>8</v>
       </c>
-      <c r="G19" s="39"/>
+      <c r="G19" s="41"/>
       <c r="H19" s="15">
         <v>3</v>
       </c>
@@ -2619,7 +2619,7 @@
       <c r="F21" s="14">
         <v>8</v>
       </c>
-      <c r="G21" s="39">
+      <c r="G21" s="41">
         <v>56</v>
       </c>
       <c r="I21" s="11" t="s">
@@ -2662,7 +2662,7 @@
       <c r="F22" s="14">
         <v>8</v>
       </c>
-      <c r="G22" s="39"/>
+      <c r="G22" s="41"/>
       <c r="I22" s="11" t="s">
         <v>49</v>
       </c>
@@ -2702,7 +2702,7 @@
       <c r="F23" s="14">
         <v>8</v>
       </c>
-      <c r="G23" s="39"/>
+      <c r="G23" s="41"/>
       <c r="K23" s="16">
         <f t="shared" ref="K23:L23" si="1">SUM(K18:K22)</f>
         <v>27</v>
@@ -2738,7 +2738,7 @@
       <c r="F24" s="14">
         <v>8</v>
       </c>
-      <c r="G24" s="39"/>
+      <c r="G24" s="41"/>
       <c r="I24" s="11"/>
       <c r="O24" s="5" t="s">
         <v>10</v>
@@ -2767,11 +2767,11 @@
       <c r="F25" s="14">
         <v>12</v>
       </c>
-      <c r="G25" s="39"/>
+      <c r="G25" s="41"/>
       <c r="H25" s="15">
         <v>4</v>
       </c>
-      <c r="I25" s="40" t="s">
+      <c r="I25" s="42" t="s">
         <v>65</v>
       </c>
       <c r="J25" s="17">
@@ -2807,11 +2807,11 @@
       <c r="F26" s="14">
         <v>12</v>
       </c>
-      <c r="G26" s="39"/>
+      <c r="G26" s="41"/>
       <c r="H26" s="15">
         <v>7</v>
       </c>
-      <c r="I26" s="40"/>
+      <c r="I26" s="42"/>
       <c r="J26" s="17">
         <v>27</v>
       </c>
@@ -2848,7 +2848,7 @@
       <c r="H27" s="15">
         <v>4</v>
       </c>
-      <c r="I27" s="40"/>
+      <c r="I27" s="42"/>
       <c r="J27" s="17">
         <v>45</v>
       </c>
@@ -3317,7 +3317,7 @@
         <v>5</v>
       </c>
       <c r="L10" s="11" t="s">
-        <v>75</v>
+        <v>84</v>
       </c>
     </row>
     <row r="11" spans="1:15" ht="15.5" x14ac:dyDescent="0.25">
@@ -3365,11 +3365,11 @@
       <c r="I12" s="29">
         <v>0</v>
       </c>
-      <c r="L12" s="41" t="s">
-        <v>76</v>
-      </c>
-      <c r="M12" s="42"/>
-      <c r="N12" s="43"/>
+      <c r="L12" s="43" t="s">
+        <v>75</v>
+      </c>
+      <c r="M12" s="44"/>
+      <c r="N12" s="45"/>
       <c r="O12" s="18" t="s">
         <v>67</v>
       </c>
@@ -3397,11 +3397,11 @@
       <c r="I13" s="32">
         <v>1</v>
       </c>
-      <c r="L13" s="44" t="s">
-        <v>77</v>
-      </c>
-      <c r="M13" s="45"/>
-      <c r="N13" s="46"/>
+      <c r="L13" s="46" t="s">
+        <v>76</v>
+      </c>
+      <c r="M13" s="47"/>
+      <c r="N13" s="48"/>
       <c r="O13" s="33">
         <v>0.19</v>
       </c>
@@ -3433,11 +3433,11 @@
         <f>J3*M2</f>
         <v>1900</v>
       </c>
-      <c r="L14" s="44" t="s">
-        <v>78</v>
-      </c>
-      <c r="M14" s="45"/>
-      <c r="N14" s="46"/>
+      <c r="L14" s="46" t="s">
+        <v>77</v>
+      </c>
+      <c r="M14" s="47"/>
+      <c r="N14" s="48"/>
       <c r="O14" s="34">
         <v>0.28499999999999998</v>
       </c>
@@ -3463,11 +3463,11 @@
       <c r="I15" s="29">
         <v>7</v>
       </c>
-      <c r="L15" s="44" t="s">
-        <v>79</v>
-      </c>
-      <c r="M15" s="45"/>
-      <c r="N15" s="46"/>
+      <c r="L15" s="46" t="s">
+        <v>78</v>
+      </c>
+      <c r="M15" s="47"/>
+      <c r="N15" s="48"/>
       <c r="O15" s="34">
         <v>0.33250000000000002</v>
       </c>
@@ -3520,7 +3520,7 @@
         <v>2</v>
       </c>
       <c r="L17" s="30" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
     </row>
     <row r="18" spans="1:12" ht="15.5" x14ac:dyDescent="0.25">
@@ -3571,7 +3571,7 @@
         <v>0</v>
       </c>
       <c r="L19" s="11" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
     </row>
     <row r="20" spans="1:12" ht="15.5" x14ac:dyDescent="0.25">
@@ -3622,7 +3622,7 @@
         <v>0</v>
       </c>
       <c r="L21" s="11" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
     </row>
     <row r="22" spans="1:12" ht="15.5" x14ac:dyDescent="0.25">
@@ -3649,7 +3649,7 @@
         <v>0</v>
       </c>
       <c r="L22" s="11" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
     </row>
     <row r="23" spans="1:12" ht="15.5" x14ac:dyDescent="0.25">
@@ -3865,8 +3865,8 @@
       <c r="C2" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="D2" s="48" t="s">
-        <v>84</v>
+      <c r="D2" s="40" t="s">
+        <v>83</v>
       </c>
       <c r="E2" s="11" t="s">
         <v>51</v>
@@ -3892,7 +3892,7 @@
       <c r="E3" s="14">
         <v>12</v>
       </c>
-      <c r="F3" s="39">
+      <c r="F3" s="41">
         <v>36</v>
       </c>
       <c r="G3" s="15">
@@ -3920,7 +3920,7 @@
       <c r="E4" s="14">
         <v>12</v>
       </c>
-      <c r="F4" s="39"/>
+      <c r="F4" s="41"/>
       <c r="G4" s="15">
         <v>4</v>
       </c>
@@ -3946,7 +3946,7 @@
       <c r="E5" s="14">
         <v>12</v>
       </c>
-      <c r="F5" s="39"/>
+      <c r="F5" s="41"/>
       <c r="G5" s="15">
         <v>7</v>
       </c>
@@ -3966,13 +3966,13 @@
       <c r="C6" s="3">
         <v>46166</v>
       </c>
-      <c r="D6" s="47" t="s">
+      <c r="D6" s="39" t="s">
         <v>7</v>
       </c>
       <c r="E6">
         <v>0</v>
       </c>
-      <c r="F6" s="39"/>
+      <c r="F6" s="41"/>
       <c r="G6" s="15"/>
       <c r="N6" s="5" t="s">
         <v>19</v>
@@ -3996,7 +3996,7 @@
       <c r="E7" s="14">
         <v>12</v>
       </c>
-      <c r="F7" s="39">
+      <c r="F7" s="41">
         <v>68</v>
       </c>
       <c r="G7" s="15">
@@ -4024,7 +4024,7 @@
       <c r="E8" s="14">
         <v>12</v>
       </c>
-      <c r="F8" s="39"/>
+      <c r="F8" s="41"/>
       <c r="G8" s="15">
         <v>4</v>
       </c>
@@ -4050,7 +4050,7 @@
       <c r="E9" s="14">
         <v>12</v>
       </c>
-      <c r="F9" s="39"/>
+      <c r="F9" s="41"/>
       <c r="G9" s="15">
         <v>4</v>
       </c>
@@ -4076,7 +4076,7 @@
       <c r="E10" s="14">
         <v>12</v>
       </c>
-      <c r="F10" s="39"/>
+      <c r="F10" s="41"/>
       <c r="G10" s="15">
         <v>4</v>
       </c>
@@ -4102,7 +4102,7 @@
       <c r="E11" s="14">
         <v>12</v>
       </c>
-      <c r="F11" s="39"/>
+      <c r="F11" s="41"/>
       <c r="G11" s="15">
         <v>4</v>
       </c>
@@ -4128,7 +4128,7 @@
       <c r="E12" s="14">
         <v>8</v>
       </c>
-      <c r="F12" s="39"/>
+      <c r="F12" s="41"/>
       <c r="G12" s="15">
         <v>3</v>
       </c>
@@ -4176,7 +4176,7 @@
       <c r="E14" s="14">
         <v>8</v>
       </c>
-      <c r="F14" s="39">
+      <c r="F14" s="41">
         <v>48</v>
       </c>
       <c r="H14" s="11" t="s">
@@ -4207,7 +4207,7 @@
       <c r="E15" s="14">
         <v>8</v>
       </c>
-      <c r="F15" s="39"/>
+      <c r="F15" s="41"/>
       <c r="N15" s="5" t="s">
         <v>28</v>
       </c>
@@ -4230,7 +4230,7 @@
       <c r="E16" s="14">
         <v>8</v>
       </c>
-      <c r="F16" s="39"/>
+      <c r="F16" s="41"/>
       <c r="N16" s="5" t="s">
         <v>29</v>
       </c>
@@ -4253,7 +4253,7 @@
       <c r="E17" s="14">
         <v>8</v>
       </c>
-      <c r="F17" s="39"/>
+      <c r="F17" s="41"/>
       <c r="I17" s="11" t="s">
         <v>50</v>
       </c>
@@ -4285,7 +4285,7 @@
       <c r="E18" s="14">
         <v>8</v>
       </c>
-      <c r="F18" s="39"/>
+      <c r="F18" s="41"/>
       <c r="H18" s="11" t="s">
         <v>45</v>
       </c>
@@ -4320,7 +4320,7 @@
       <c r="E19" s="14">
         <v>8</v>
       </c>
-      <c r="F19" s="39"/>
+      <c r="F19" s="41"/>
       <c r="G19" s="15">
         <v>3</v>
       </c>
@@ -4392,7 +4392,7 @@
       <c r="E21" s="14">
         <v>8</v>
       </c>
-      <c r="F21" s="39">
+      <c r="F21" s="41">
         <v>56</v>
       </c>
       <c r="H21" s="11" t="s">
@@ -4430,7 +4430,7 @@
       <c r="E22" s="14">
         <v>8</v>
       </c>
-      <c r="F22" s="39"/>
+      <c r="F22" s="41"/>
       <c r="H22" s="11" t="s">
         <v>49</v>
       </c>
@@ -4465,7 +4465,7 @@
       <c r="E23" s="14">
         <v>8</v>
       </c>
-      <c r="F23" s="39"/>
+      <c r="F23" s="41"/>
       <c r="J23" s="16">
         <f t="shared" ref="J23:K23" si="1">SUM(J18:J22)</f>
         <v>27</v>
@@ -4496,7 +4496,7 @@
       <c r="E24" s="14">
         <v>8</v>
       </c>
-      <c r="F24" s="39"/>
+      <c r="F24" s="41"/>
       <c r="H24" s="11"/>
       <c r="N24" s="5" t="s">
         <v>10</v>
@@ -4520,11 +4520,11 @@
       <c r="E25" s="14">
         <v>12</v>
       </c>
-      <c r="F25" s="39"/>
+      <c r="F25" s="41"/>
       <c r="G25" s="15">
         <v>4</v>
       </c>
-      <c r="H25" s="40" t="s">
+      <c r="H25" s="42" t="s">
         <v>65</v>
       </c>
       <c r="I25" s="17">
@@ -4555,11 +4555,11 @@
       <c r="E26" s="14">
         <v>12</v>
       </c>
-      <c r="F26" s="39"/>
+      <c r="F26" s="41"/>
       <c r="G26" s="15">
         <v>7</v>
       </c>
-      <c r="H26" s="40"/>
+      <c r="H26" s="42"/>
       <c r="I26" s="17">
         <v>27</v>
       </c>
@@ -4591,7 +4591,7 @@
       <c r="G27" s="15">
         <v>4</v>
       </c>
-      <c r="H27" s="40"/>
+      <c r="H27" s="42"/>
       <c r="I27" s="17">
         <v>45</v>
       </c>
@@ -4744,7 +4744,7 @@
     <mergeCell ref="F21:F26"/>
     <mergeCell ref="H25:H27"/>
   </mergeCells>
-  <conditionalFormatting sqref="B3:B31 B33 A32:B32 D32">
+  <conditionalFormatting sqref="B3:B31 A32:B32 D32 B33">
     <cfRule type="containsText" dxfId="0" priority="1" operator="containsText" text="dimanche">
       <formula>NOT(ISERROR(SEARCH("dimanche",A3)))</formula>
     </cfRule>

</xml_diff>

<commit_message>
Mise à jour du 05 oct 2026
</commit_message>
<xml_diff>
--- a/HS & COMPLEMENT CSKN.xlsx
+++ b/HS & COMPLEMENT CSKN.xlsx
@@ -10,7 +10,7 @@
   </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CE970697-2834-4AE1-BA67-8BEB194FFD90}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28690" yWindow="-110" windowWidth="29020" windowHeight="15700" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" firstSheet="1" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Esprit Sucrière (HS)" sheetId="1" r:id="rId1"/>
@@ -541,12 +541,6 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -564,6 +558,12 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -984,7 +984,7 @@
       <c r="F3" s="14">
         <v>12</v>
       </c>
-      <c r="G3" s="41">
+      <c r="G3" s="47">
         <v>36</v>
       </c>
       <c r="H3" s="15">
@@ -1017,7 +1017,7 @@
       <c r="F4" s="14">
         <v>12</v>
       </c>
-      <c r="G4" s="41"/>
+      <c r="G4" s="47"/>
       <c r="H4" s="15">
         <v>4</v>
       </c>
@@ -1048,7 +1048,7 @@
       <c r="F5" s="14">
         <v>12</v>
       </c>
-      <c r="G5" s="41"/>
+      <c r="G5" s="47"/>
       <c r="H5" s="15">
         <v>4</v>
       </c>
@@ -1083,7 +1083,7 @@
       <c r="F6">
         <v>0</v>
       </c>
-      <c r="G6" s="41"/>
+      <c r="G6" s="47"/>
       <c r="H6" s="15"/>
       <c r="I6" s="18" t="s">
         <v>40</v>
@@ -1118,7 +1118,7 @@
       <c r="F7" s="14">
         <v>12</v>
       </c>
-      <c r="G7" s="41">
+      <c r="G7" s="47">
         <v>68</v>
       </c>
       <c r="H7" s="15">
@@ -1157,7 +1157,7 @@
       <c r="F8" s="14">
         <v>12</v>
       </c>
-      <c r="G8" s="41"/>
+      <c r="G8" s="47"/>
       <c r="H8" s="15">
         <v>4</v>
       </c>
@@ -1194,7 +1194,7 @@
       <c r="F9" s="14">
         <v>12</v>
       </c>
-      <c r="G9" s="41"/>
+      <c r="G9" s="47"/>
       <c r="H9" s="15">
         <v>4</v>
       </c>
@@ -1231,7 +1231,7 @@
       <c r="F10" s="14">
         <v>12</v>
       </c>
-      <c r="G10" s="41"/>
+      <c r="G10" s="47"/>
       <c r="H10" s="15">
         <v>4</v>
       </c>
@@ -1268,7 +1268,7 @@
       <c r="F11" s="14">
         <v>12</v>
       </c>
-      <c r="G11" s="41"/>
+      <c r="G11" s="47"/>
       <c r="H11" s="15">
         <v>4</v>
       </c>
@@ -1299,7 +1299,7 @@
       <c r="F12" s="14">
         <v>8</v>
       </c>
-      <c r="G12" s="41"/>
+      <c r="G12" s="47"/>
       <c r="H12" s="15"/>
       <c r="O12" s="5" t="s">
         <v>25</v>
@@ -1355,7 +1355,7 @@
       <c r="F14" s="14">
         <v>8</v>
       </c>
-      <c r="G14" s="41">
+      <c r="G14" s="47">
         <v>48</v>
       </c>
       <c r="I14" s="11" t="s">
@@ -1389,7 +1389,7 @@
       <c r="F15" s="14">
         <v>8</v>
       </c>
-      <c r="G15" s="41"/>
+      <c r="G15" s="47"/>
       <c r="I15" s="11" t="s">
         <v>64</v>
       </c>
@@ -1420,7 +1420,7 @@
       <c r="F16" s="14">
         <v>8</v>
       </c>
-      <c r="G16" s="41"/>
+      <c r="G16" s="47"/>
       <c r="O16" s="5" t="s">
         <v>29</v>
       </c>
@@ -1448,7 +1448,7 @@
       <c r="F17" s="14">
         <v>8</v>
       </c>
-      <c r="G17" s="41"/>
+      <c r="G17" s="47"/>
       <c r="I17" s="17"/>
       <c r="J17" s="19" t="s">
         <v>59</v>
@@ -1489,7 +1489,7 @@
       <c r="F18" s="14">
         <v>8</v>
       </c>
-      <c r="G18" s="41"/>
+      <c r="G18" s="47"/>
       <c r="I18" s="18" t="s">
         <v>58</v>
       </c>
@@ -1532,7 +1532,7 @@
       <c r="F19" s="14">
         <v>8</v>
       </c>
-      <c r="G19" s="41"/>
+      <c r="G19" s="47"/>
       <c r="I19" s="11"/>
       <c r="O19" s="5" t="s">
         <v>32</v>
@@ -1589,10 +1589,10 @@
       <c r="F21" s="14">
         <v>8</v>
       </c>
-      <c r="G21" s="41">
+      <c r="G21" s="47">
         <v>56</v>
       </c>
-      <c r="I21" s="42" t="s">
+      <c r="I21" s="48" t="s">
         <v>62</v>
       </c>
       <c r="J21" s="17">
@@ -1630,8 +1630,8 @@
       <c r="F22" s="14">
         <v>8</v>
       </c>
-      <c r="G22" s="41"/>
-      <c r="I22" s="42"/>
+      <c r="G22" s="47"/>
+      <c r="I22" s="48"/>
       <c r="J22" s="17">
         <v>24</v>
       </c>
@@ -1665,8 +1665,8 @@
       <c r="F23" s="14">
         <v>8</v>
       </c>
-      <c r="G23" s="41"/>
-      <c r="I23" s="42"/>
+      <c r="G23" s="47"/>
+      <c r="I23" s="48"/>
       <c r="J23" s="17">
         <v>36</v>
       </c>
@@ -1700,7 +1700,7 @@
       <c r="F24" s="14">
         <v>8</v>
       </c>
-      <c r="G24" s="41"/>
+      <c r="G24" s="47"/>
       <c r="O24" s="5" t="s">
         <v>10</v>
       </c>
@@ -1728,7 +1728,7 @@
       <c r="F25" s="14">
         <v>12</v>
       </c>
-      <c r="G25" s="41"/>
+      <c r="G25" s="47"/>
       <c r="H25" s="15">
         <v>4</v>
       </c>
@@ -1759,7 +1759,7 @@
       <c r="F26" s="14">
         <v>12</v>
       </c>
-      <c r="G26" s="41"/>
+      <c r="G26" s="47"/>
       <c r="H26" s="15">
         <v>4</v>
       </c>
@@ -2031,7 +2031,7 @@
       <c r="F3" s="14">
         <v>12</v>
       </c>
-      <c r="G3" s="41">
+      <c r="G3" s="47">
         <v>36</v>
       </c>
       <c r="H3" s="15">
@@ -2064,7 +2064,7 @@
       <c r="F4" s="14">
         <v>12</v>
       </c>
-      <c r="G4" s="41"/>
+      <c r="G4" s="47"/>
       <c r="H4" s="15">
         <v>4</v>
       </c>
@@ -2095,7 +2095,7 @@
       <c r="F5" s="14">
         <v>12</v>
       </c>
-      <c r="G5" s="41"/>
+      <c r="G5" s="47"/>
       <c r="H5" s="15">
         <v>7</v>
       </c>
@@ -2124,7 +2124,7 @@
       <c r="F6">
         <v>0</v>
       </c>
-      <c r="G6" s="41"/>
+      <c r="G6" s="47"/>
       <c r="H6" s="15"/>
       <c r="O6" s="5" t="s">
         <v>19</v>
@@ -2153,7 +2153,7 @@
       <c r="F7" s="14">
         <v>12</v>
       </c>
-      <c r="G7" s="41">
+      <c r="G7" s="47">
         <v>68</v>
       </c>
       <c r="H7" s="15">
@@ -2186,7 +2186,7 @@
       <c r="F8" s="14">
         <v>12</v>
       </c>
-      <c r="G8" s="41"/>
+      <c r="G8" s="47"/>
       <c r="H8" s="15">
         <v>4</v>
       </c>
@@ -2217,7 +2217,7 @@
       <c r="F9" s="14">
         <v>12</v>
       </c>
-      <c r="G9" s="41"/>
+      <c r="G9" s="47"/>
       <c r="H9" s="15">
         <v>4</v>
       </c>
@@ -2248,7 +2248,7 @@
       <c r="F10" s="14">
         <v>12</v>
       </c>
-      <c r="G10" s="41"/>
+      <c r="G10" s="47"/>
       <c r="H10" s="15">
         <v>4</v>
       </c>
@@ -2279,7 +2279,7 @@
       <c r="F11" s="14">
         <v>12</v>
       </c>
-      <c r="G11" s="41"/>
+      <c r="G11" s="47"/>
       <c r="H11" s="15">
         <v>4</v>
       </c>
@@ -2310,7 +2310,7 @@
       <c r="F12" s="14">
         <v>8</v>
       </c>
-      <c r="G12" s="41"/>
+      <c r="G12" s="47"/>
       <c r="H12" s="15">
         <v>3</v>
       </c>
@@ -2368,7 +2368,7 @@
       <c r="F14" s="14">
         <v>8</v>
       </c>
-      <c r="G14" s="41">
+      <c r="G14" s="47">
         <v>48</v>
       </c>
       <c r="I14" s="11" t="s">
@@ -2404,7 +2404,7 @@
       <c r="F15" s="14">
         <v>8</v>
       </c>
-      <c r="G15" s="41"/>
+      <c r="G15" s="47"/>
       <c r="O15" s="5" t="s">
         <v>28</v>
       </c>
@@ -2432,7 +2432,7 @@
       <c r="F16" s="14">
         <v>8</v>
       </c>
-      <c r="G16" s="41"/>
+      <c r="G16" s="47"/>
       <c r="O16" s="5" t="s">
         <v>29</v>
       </c>
@@ -2460,7 +2460,7 @@
       <c r="F17" s="14">
         <v>8</v>
       </c>
-      <c r="G17" s="41"/>
+      <c r="G17" s="47"/>
       <c r="J17" s="11" t="s">
         <v>50</v>
       </c>
@@ -2497,7 +2497,7 @@
       <c r="F18" s="14">
         <v>8</v>
       </c>
-      <c r="G18" s="41"/>
+      <c r="G18" s="47"/>
       <c r="I18" s="11" t="s">
         <v>45</v>
       </c>
@@ -2537,7 +2537,7 @@
       <c r="F19" s="14">
         <v>8</v>
       </c>
-      <c r="G19" s="41"/>
+      <c r="G19" s="47"/>
       <c r="H19" s="15">
         <v>3</v>
       </c>
@@ -2619,7 +2619,7 @@
       <c r="F21" s="14">
         <v>8</v>
       </c>
-      <c r="G21" s="41">
+      <c r="G21" s="47">
         <v>56</v>
       </c>
       <c r="I21" s="11" t="s">
@@ -2662,7 +2662,7 @@
       <c r="F22" s="14">
         <v>8</v>
       </c>
-      <c r="G22" s="41"/>
+      <c r="G22" s="47"/>
       <c r="I22" s="11" t="s">
         <v>49</v>
       </c>
@@ -2702,7 +2702,7 @@
       <c r="F23" s="14">
         <v>8</v>
       </c>
-      <c r="G23" s="41"/>
+      <c r="G23" s="47"/>
       <c r="K23" s="16">
         <f t="shared" ref="K23:L23" si="1">SUM(K18:K22)</f>
         <v>27</v>
@@ -2738,7 +2738,7 @@
       <c r="F24" s="14">
         <v>8</v>
       </c>
-      <c r="G24" s="41"/>
+      <c r="G24" s="47"/>
       <c r="I24" s="11"/>
       <c r="O24" s="5" t="s">
         <v>10</v>
@@ -2767,11 +2767,11 @@
       <c r="F25" s="14">
         <v>12</v>
       </c>
-      <c r="G25" s="41"/>
+      <c r="G25" s="47"/>
       <c r="H25" s="15">
         <v>4</v>
       </c>
-      <c r="I25" s="42" t="s">
+      <c r="I25" s="48" t="s">
         <v>65</v>
       </c>
       <c r="J25" s="17">
@@ -2807,11 +2807,11 @@
       <c r="F26" s="14">
         <v>12</v>
       </c>
-      <c r="G26" s="41"/>
+      <c r="G26" s="47"/>
       <c r="H26" s="15">
         <v>7</v>
       </c>
-      <c r="I26" s="42"/>
+      <c r="I26" s="48"/>
       <c r="J26" s="17">
         <v>27</v>
       </c>
@@ -2848,7 +2848,7 @@
       <c r="H27" s="15">
         <v>4</v>
       </c>
-      <c r="I27" s="42"/>
+      <c r="I27" s="48"/>
       <c r="J27" s="17">
         <v>45</v>
       </c>
@@ -3365,11 +3365,11 @@
       <c r="I12" s="29">
         <v>0</v>
       </c>
-      <c r="L12" s="43" t="s">
+      <c r="L12" s="41" t="s">
         <v>75</v>
       </c>
-      <c r="M12" s="44"/>
-      <c r="N12" s="45"/>
+      <c r="M12" s="42"/>
+      <c r="N12" s="43"/>
       <c r="O12" s="18" t="s">
         <v>67</v>
       </c>
@@ -3397,11 +3397,11 @@
       <c r="I13" s="32">
         <v>1</v>
       </c>
-      <c r="L13" s="46" t="s">
+      <c r="L13" s="44" t="s">
         <v>76</v>
       </c>
-      <c r="M13" s="47"/>
-      <c r="N13" s="48"/>
+      <c r="M13" s="45"/>
+      <c r="N13" s="46"/>
       <c r="O13" s="33">
         <v>0.19</v>
       </c>
@@ -3433,11 +3433,11 @@
         <f>J3*M2</f>
         <v>1900</v>
       </c>
-      <c r="L14" s="46" t="s">
+      <c r="L14" s="44" t="s">
         <v>77</v>
       </c>
-      <c r="M14" s="47"/>
-      <c r="N14" s="48"/>
+      <c r="M14" s="45"/>
+      <c r="N14" s="46"/>
       <c r="O14" s="34">
         <v>0.28499999999999998</v>
       </c>
@@ -3463,11 +3463,11 @@
       <c r="I15" s="29">
         <v>7</v>
       </c>
-      <c r="L15" s="46" t="s">
+      <c r="L15" s="44" t="s">
         <v>78</v>
       </c>
-      <c r="M15" s="47"/>
-      <c r="N15" s="48"/>
+      <c r="M15" s="45"/>
+      <c r="N15" s="46"/>
       <c r="O15" s="34">
         <v>0.33250000000000002</v>
       </c>
@@ -3892,7 +3892,7 @@
       <c r="E3" s="14">
         <v>12</v>
       </c>
-      <c r="F3" s="41">
+      <c r="F3" s="47">
         <v>36</v>
       </c>
       <c r="G3" s="15">
@@ -3920,7 +3920,7 @@
       <c r="E4" s="14">
         <v>12</v>
       </c>
-      <c r="F4" s="41"/>
+      <c r="F4" s="47"/>
       <c r="G4" s="15">
         <v>4</v>
       </c>
@@ -3946,7 +3946,7 @@
       <c r="E5" s="14">
         <v>12</v>
       </c>
-      <c r="F5" s="41"/>
+      <c r="F5" s="47"/>
       <c r="G5" s="15">
         <v>7</v>
       </c>
@@ -3972,7 +3972,7 @@
       <c r="E6">
         <v>0</v>
       </c>
-      <c r="F6" s="41"/>
+      <c r="F6" s="47"/>
       <c r="G6" s="15"/>
       <c r="N6" s="5" t="s">
         <v>19</v>
@@ -3996,7 +3996,7 @@
       <c r="E7" s="14">
         <v>12</v>
       </c>
-      <c r="F7" s="41">
+      <c r="F7" s="47">
         <v>68</v>
       </c>
       <c r="G7" s="15">
@@ -4024,7 +4024,7 @@
       <c r="E8" s="14">
         <v>12</v>
       </c>
-      <c r="F8" s="41"/>
+      <c r="F8" s="47"/>
       <c r="G8" s="15">
         <v>4</v>
       </c>
@@ -4050,7 +4050,7 @@
       <c r="E9" s="14">
         <v>12</v>
       </c>
-      <c r="F9" s="41"/>
+      <c r="F9" s="47"/>
       <c r="G9" s="15">
         <v>4</v>
       </c>
@@ -4076,7 +4076,7 @@
       <c r="E10" s="14">
         <v>12</v>
       </c>
-      <c r="F10" s="41"/>
+      <c r="F10" s="47"/>
       <c r="G10" s="15">
         <v>4</v>
       </c>
@@ -4102,7 +4102,7 @@
       <c r="E11" s="14">
         <v>12</v>
       </c>
-      <c r="F11" s="41"/>
+      <c r="F11" s="47"/>
       <c r="G11" s="15">
         <v>4</v>
       </c>
@@ -4128,7 +4128,7 @@
       <c r="E12" s="14">
         <v>8</v>
       </c>
-      <c r="F12" s="41"/>
+      <c r="F12" s="47"/>
       <c r="G12" s="15">
         <v>3</v>
       </c>
@@ -4176,7 +4176,7 @@
       <c r="E14" s="14">
         <v>8</v>
       </c>
-      <c r="F14" s="41">
+      <c r="F14" s="47">
         <v>48</v>
       </c>
       <c r="H14" s="11" t="s">
@@ -4207,7 +4207,7 @@
       <c r="E15" s="14">
         <v>8</v>
       </c>
-      <c r="F15" s="41"/>
+      <c r="F15" s="47"/>
       <c r="N15" s="5" t="s">
         <v>28</v>
       </c>
@@ -4230,7 +4230,7 @@
       <c r="E16" s="14">
         <v>8</v>
       </c>
-      <c r="F16" s="41"/>
+      <c r="F16" s="47"/>
       <c r="N16" s="5" t="s">
         <v>29</v>
       </c>
@@ -4253,7 +4253,7 @@
       <c r="E17" s="14">
         <v>8</v>
       </c>
-      <c r="F17" s="41"/>
+      <c r="F17" s="47"/>
       <c r="I17" s="11" t="s">
         <v>50</v>
       </c>
@@ -4285,7 +4285,7 @@
       <c r="E18" s="14">
         <v>8</v>
       </c>
-      <c r="F18" s="41"/>
+      <c r="F18" s="47"/>
       <c r="H18" s="11" t="s">
         <v>45</v>
       </c>
@@ -4320,7 +4320,7 @@
       <c r="E19" s="14">
         <v>8</v>
       </c>
-      <c r="F19" s="41"/>
+      <c r="F19" s="47"/>
       <c r="G19" s="15">
         <v>3</v>
       </c>
@@ -4392,7 +4392,7 @@
       <c r="E21" s="14">
         <v>8</v>
       </c>
-      <c r="F21" s="41">
+      <c r="F21" s="47">
         <v>56</v>
       </c>
       <c r="H21" s="11" t="s">
@@ -4430,7 +4430,7 @@
       <c r="E22" s="14">
         <v>8</v>
       </c>
-      <c r="F22" s="41"/>
+      <c r="F22" s="47"/>
       <c r="H22" s="11" t="s">
         <v>49</v>
       </c>
@@ -4465,7 +4465,7 @@
       <c r="E23" s="14">
         <v>8</v>
       </c>
-      <c r="F23" s="41"/>
+      <c r="F23" s="47"/>
       <c r="J23" s="16">
         <f t="shared" ref="J23:K23" si="1">SUM(J18:J22)</f>
         <v>27</v>
@@ -4496,7 +4496,7 @@
       <c r="E24" s="14">
         <v>8</v>
       </c>
-      <c r="F24" s="41"/>
+      <c r="F24" s="47"/>
       <c r="H24" s="11"/>
       <c r="N24" s="5" t="s">
         <v>10</v>
@@ -4520,11 +4520,11 @@
       <c r="E25" s="14">
         <v>12</v>
       </c>
-      <c r="F25" s="41"/>
+      <c r="F25" s="47"/>
       <c r="G25" s="15">
         <v>4</v>
       </c>
-      <c r="H25" s="42" t="s">
+      <c r="H25" s="48" t="s">
         <v>65</v>
       </c>
       <c r="I25" s="17">
@@ -4555,11 +4555,11 @@
       <c r="E26" s="14">
         <v>12</v>
       </c>
-      <c r="F26" s="41"/>
+      <c r="F26" s="47"/>
       <c r="G26" s="15">
         <v>7</v>
       </c>
-      <c r="H26" s="42"/>
+      <c r="H26" s="48"/>
       <c r="I26" s="17">
         <v>27</v>
       </c>
@@ -4591,7 +4591,7 @@
       <c r="G27" s="15">
         <v>4</v>
       </c>
-      <c r="H27" s="42"/>
+      <c r="H27" s="48"/>
       <c r="I27" s="17">
         <v>45</v>
       </c>

</xml_diff>